<commit_message>
feat: close out 114 with rankings + 114 新申請 recipients, pre-create 匯入 accounts
- 造冊管理 114-整學年 showed 無法載入學生資料: the matrix preview/roster
  path joins allocated CollegeRankingItems and raised because no finalized,
  distribution-executed ranking existed. Seed one ranking per college
  (C/E) for 113 and 114 with the year's 新申請 as allocated items, and add
  two 114 新申請得獎者 (114新申請- prefix) so 114 has ranked recipients, not
  only renewals. Rosters now reference their ranking; approved apps carry
  quota_allocation_status/review_stage/approved_at as finalize sets them.
- 批次匯入 students get an account (no application) so they appear in the
  Development Login picker; the import still creates their applications.
- Mock SIS + 續領 workbook include the two 114 recipients (是/通過).

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NYWYzgwV9y9wWYJfsQ27SP
</commit_message>
<xml_diff>
--- a/docs/samples/ay115/115_續領生匯入.xlsx
+++ b/docs/samples/ay115/115_續領生匯入.xlsx
@@ -423,13 +423,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L6"/>
+  <dimension ref="A1:L8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
     <col width="10" customWidth="1" min="2" max="2"/>
     <col width="22" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="4" max="4"/>
     <col width="11" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="18" customWidth="1" min="7" max="7"/>
@@ -790,6 +790,126 @@
       <c r="K6" t="inlineStr"/>
       <c r="L6" t="inlineStr"/>
     </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>6</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>資訊學院</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>資訊科學與工程研究所</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>114新申請-何冠廷</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>314551206</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>博二</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>國科會</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>0021314551206</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>cs_professor</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>李資訊教授</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>7</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>電機學院</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>電機工程學系</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>114新申請-謝宜庭</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>314551207</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>博二</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>是</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>通過</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>教育部</t>
+        </is>
+      </c>
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>0021314551207</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>professor</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>李教授</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
chore(seed): label the 113 cohort as 113續領生; no 115 renewal for the ceiling student
- Display names of the renewal cohort read「113續領生-林承翰」 instead of
  「續領-林承翰」 in the seed, the mock SIS and the sample workbooks, so every
  roster / list makes the awarding year visible (std_cname must match across
  the three, or SIS verification fails).
- 鄭宇軒 (311551205) sits at the 36-month ceiling by 114 and the 續領 sheet marks
  them 領獎期滿 — the seed no longer creates a 115 renewal for them, so
  phd_113's 115 segment estimates 4, matching the sample's four 通過 rows.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WFuJ3GmbekmqvgTL8voLFw
</commit_message>
<xml_diff>
--- a/docs/samples/ay115/115_續領生匯入.xlsx
+++ b/docs/samples/ay115/115_續領生匯入.xlsx
@@ -518,7 +518,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>續領-林承翰</t>
+          <t>113續領生-林承翰</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -578,7 +578,7 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>續領-張雅婷</t>
+          <t>113續領生-張雅婷</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>續領-黃冠宇</t>
+          <t>113續領生-黃冠宇</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -698,7 +698,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>續領-吳佩珊</t>
+          <t>113續領生-吳佩珊</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
@@ -758,7 +758,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>續領-鄭宇軒</t>
+          <t>113續領生-鄭宇軒</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">

</xml_diff>

<commit_message>
chore(seed): name demo students by their cohort — 113續領生-… / 114續領生-…
The name prefix now says which configuration's 續領生 a demo student is:
「113續領生-林承翰」 (113 awardee, renewing in 114 and 115 on phd_113) and
「114續領生-何冠廷」 (114 awardee, renewing in 115 on phd_114), replacing the
ambiguous 「續領-」 / 「114新申請-」. Mirrored in mock-student-api, the
匯入續領生 sample workbook, and the seed summary printout.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WFuJ3GmbekmqvgTL8voLFw
</commit_message>
<xml_diff>
--- a/docs/samples/ay115/115_續領生匯入.xlsx
+++ b/docs/samples/ay115/115_續領生匯入.xlsx
@@ -806,7 +806,7 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>114新申請-何冠廷</t>
+          <t>114續領生-何冠廷</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
@@ -866,7 +866,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>114新申請-謝宜庭</t>
+          <t>114續領生-謝宜庭</t>
         </is>
       </c>
       <c r="E8" s="2" t="inlineStr">

</xml_diff>